<commit_message>
Update ICICI report + model files (REDUCE)
</commit_message>
<xml_diff>
--- a/assets/files/icici-financial-model.xlsx
+++ b/assets/files/icici-financial-model.xlsx
@@ -1464,7 +1464,6 @@
       <c r="E6" s="169" t="n"/>
       <c r="F6" s="169" t="n"/>
     </row>
-    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="68">
       <c r="B8" s="170" t="inlineStr">
         <is>
@@ -1472,7 +1471,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="15" customHeight="1" s="68">
       <c r="A10" s="171" t="inlineStr">
         <is>
@@ -1562,8 +1560,6 @@
         <v/>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="68">
       <c r="A20" s="171" t="inlineStr">
         <is>
@@ -1618,8 +1614,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
     <row r="29" ht="15" customHeight="1" s="68">
       <c r="B29" s="170" t="inlineStr">
         <is>
@@ -1719,11 +1713,11 @@
     <row r="5" ht="15" customHeight="1" s="68">
       <c r="A5" s="187" t="inlineStr">
         <is>
-          <t>Current share price (₹, 06-May-2026)</t>
+          <t>Current share price (₹, 03-Jul-2026)</t>
         </is>
       </c>
       <c r="B5" s="188" t="n">
-        <v>1280</v>
+        <v>1411.4</v>
       </c>
       <c r="C5" s="90" t="n"/>
       <c r="D5" s="90" t="n"/>
@@ -4971,7 +4965,7 @@
         </is>
       </c>
       <c r="B5" s="188" t="n">
-        <v>1280</v>
+        <v>1411.4</v>
       </c>
       <c r="C5" s="188" t="n">
         <v>75.70999999999999</v>
@@ -4998,7 +4992,7 @@
         </is>
       </c>
       <c r="B6" s="188" t="n">
-        <v>747.05</v>
+        <v>784.9</v>
       </c>
       <c r="C6" s="188" t="n">
         <v>49.39</v>
@@ -5093,8 +5087,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="236" t="inlineStr">
         <is>
@@ -5141,7 +5133,6 @@
         <v/>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="236" t="inlineStr">
         <is>
@@ -5248,7 +5239,6 @@
         <v/>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="247" t="inlineStr">
         <is>

</xml_diff>